<commit_message>
sessao 032: atualizacao rastreio colo (2016/2025) e refinamento de governanca de escrita
</commit_message>
<xml_diff>
--- a/Tools/Dashboard EMED 2026.xlsx
+++ b/Tools/Dashboard EMED 2026.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2196" uniqueCount="360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2199" uniqueCount="360">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -2210,8 +2210,8 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="2020730963"/>
-        <c:axId val="2100630040"/>
+        <c:axId val="1411506965"/>
+        <c:axId val="552247723"/>
       </c:barChart>
       <c:lineChart>
         <c:ser>
@@ -2312,11 +2312,11 @@
           </c:val>
           <c:smooth val="0"/>
         </c:ser>
-        <c:axId val="2020730963"/>
-        <c:axId val="2100630040"/>
+        <c:axId val="1411506965"/>
+        <c:axId val="552247723"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2020730963"/>
+        <c:axId val="1411506965"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2368,10 +2368,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2100630040"/>
+        <c:crossAx val="552247723"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2100630040"/>
+        <c:axId val="552247723"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2435,7 +2435,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2020730963"/>
+        <c:crossAx val="1411506965"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2616,11 +2616,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="742321468"/>
-        <c:axId val="1344586004"/>
+        <c:axId val="26604705"/>
+        <c:axId val="1292236289"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="742321468"/>
+        <c:axId val="26604705"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2672,10 +2672,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1344586004"/>
+        <c:crossAx val="1292236289"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1344586004"/>
+        <c:axId val="1292236289"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2739,7 +2739,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="742321468"/>
+        <c:crossAx val="26604705"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -2902,11 +2902,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="484058536"/>
-        <c:axId val="1392964210"/>
+        <c:axId val="1210698446"/>
+        <c:axId val="1326518910"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="484058536"/>
+        <c:axId val="1210698446"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2958,10 +2958,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1392964210"/>
+        <c:crossAx val="1326518910"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1392964210"/>
+        <c:axId val="1326518910"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3025,7 +3025,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="484058536"/>
+        <c:crossAx val="1210698446"/>
       </c:valAx>
     </c:plotArea>
     <c:plotVisOnly val="1"/>
@@ -21043,19 +21043,19 @@
       </c>
       <c r="C5" s="11">
         <f>Pediatria!E101</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D5" s="12">
         <f>'Quadro Geral'!$C5/97</f>
-        <v>0.07216494845</v>
+        <v>0.0824742268</v>
       </c>
       <c r="E5" s="13">
         <f>Pediatria!F101</f>
-        <v>192</v>
+        <v>220</v>
       </c>
       <c r="F5" s="14">
         <f>Pediatria!H101</f>
-        <v>0.796875</v>
+        <v>0.8227272727</v>
       </c>
     </row>
     <row r="6">
@@ -21106,19 +21106,19 @@
       </c>
       <c r="C8" s="16">
         <f>Preventiva!E91</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="17">
         <f>Preventiva!E91/87</f>
-        <v>0.09195402299</v>
+        <v>0.1034482759</v>
       </c>
       <c r="E8" s="18">
         <f>Preventiva!F91</f>
-        <v>309</v>
+        <v>343</v>
       </c>
       <c r="F8" s="19">
         <f>Preventiva!H91</f>
-        <v>0.7799352751</v>
+        <v>0.8017492711</v>
       </c>
     </row>
     <row r="9">
@@ -21169,19 +21169,19 @@
       </c>
       <c r="C11" s="11">
         <f>Gastro!E35</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D11" s="20">
         <f>Gastro!E35/31</f>
-        <v>0.06451612903</v>
+        <v>0.09677419355</v>
       </c>
       <c r="E11" s="18">
         <f>Gastro!F35</f>
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="F11" s="19">
         <f>Gastro!H35</f>
-        <v>0.7820512821</v>
+        <v>0.7669902913</v>
       </c>
     </row>
     <row r="12">
@@ -21463,15 +21463,15 @@
       </c>
       <c r="C25" s="23">
         <f>SUM(C5:C24)</f>
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D25" s="24">
         <f>SUM(D5:D24)/20</f>
-        <v>0.06030790361</v>
+        <v>0.06301098339</v>
       </c>
       <c r="E25" s="22">
         <f>SUM(E5:E24)</f>
-        <v>1964</v>
+        <v>2051</v>
       </c>
       <c r="F25" s="25" t="str">
         <f>#REF!/'Quadro Geral'!$E25</f>
@@ -33988,12 +33988,18 @@
       <c r="D15" s="22" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="49"/>
-      <c r="F15" s="49"/>
-      <c r="G15" s="49"/>
-      <c r="H15" s="25" t="str">
+      <c r="E15" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="53">
+        <v>28.0</v>
+      </c>
+      <c r="G15" s="53">
+        <v>28.0</v>
+      </c>
+      <c r="H15" s="25">
         <f>Pediatria!$G15/Pediatria!$F15</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -35567,19 +35573,19 @@
       <c r="D101" s="54"/>
       <c r="E101" s="22">
         <f>COUNTA(E4:E100)</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F101" s="22">
         <f t="shared" ref="F101:G101" si="1">SUM(F4:F100)</f>
-        <v>192</v>
+        <v>220</v>
       </c>
       <c r="G101" s="22">
         <f t="shared" si="1"/>
-        <v>153</v>
+        <v>181</v>
       </c>
       <c r="H101" s="25">
         <f>Pediatria!$G101/Pediatria!$F101</f>
-        <v>0.796875</v>
+        <v>0.8227272727</v>
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1">
@@ -36847,12 +36853,18 @@
       <c r="D15" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="25" t="str">
+      <c r="E15" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="53">
+        <v>34.0</v>
+      </c>
+      <c r="G15" s="53">
+        <v>34.0</v>
+      </c>
+      <c r="H15" s="25">
         <f>Preventiva!$G15/Preventiva!$F15</f>
-        <v>#DIV/0!</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -38237,19 +38249,19 @@
       <c r="D91" s="54"/>
       <c r="E91" s="22">
         <f>COUNTA(E4:E90)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F91" s="22">
         <f t="shared" ref="F91:G91" si="1">SUM(F4:F90)</f>
-        <v>309</v>
+        <v>343</v>
       </c>
       <c r="G91" s="22">
         <f t="shared" si="1"/>
-        <v>241</v>
+        <v>275</v>
       </c>
       <c r="H91" s="25">
         <f>Preventiva!$G91/Preventiva!$F91</f>
-        <v>0.7799352751</v>
+        <v>0.8017492711</v>
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
@@ -48416,12 +48428,18 @@
       <c r="D10" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="25" t="str">
+      <c r="E10" s="53" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="53">
+        <v>25.0</v>
+      </c>
+      <c r="G10" s="53">
+        <v>18.0</v>
+      </c>
+      <c r="H10" s="25">
         <f>Gastro!$G10/Gastro!$F10</f>
-        <v>#DIV/0!</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="11">
@@ -48876,19 +48894,19 @@
       <c r="D35" s="54"/>
       <c r="E35" s="22">
         <f>COUNTA(E4:E34)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F35" s="22">
         <f t="shared" ref="F35:G35" si="1">SUM(F4:F34)</f>
-        <v>78</v>
+        <v>103</v>
       </c>
       <c r="G35" s="22">
         <f t="shared" si="1"/>
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="H35" s="25">
         <f>Gastro!$G35/Gastro!$F35</f>
-        <v>0.7820512821</v>
+        <v>0.7669902913</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">

</xml_diff>